<commit_message>
Update Ferragro backend/frontend features and production docs
Align API, frontend behavior, CI/workflows, and operational documentation for the latest production deployment cycle.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/req_trabajo.xlsx
+++ b/docs/req_trabajo.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30110"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30125"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{88C5441A-3E3E-43E0-BCF9-42C502C997C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{B628F6EC-CC22-448E-A185-D2A5CAFD23A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -60,7 +60,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="662" uniqueCount="368">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="622" uniqueCount="335">
   <si>
     <t>Portal de citas de entrega Ferragro</t>
   </si>
@@ -986,181 +986,82 @@
     <t>Estudio de viabilidad</t>
   </si>
   <si>
-    <t>2026-04-22</t>
-  </si>
-  <si>
-    <t>2026-04-24</t>
-  </si>
-  <si>
     <t>Completado</t>
   </si>
   <si>
     <t>Levantamiento de requerimientos</t>
   </si>
   <si>
-    <t>2026-04-28</t>
-  </si>
-  <si>
     <t>Documentación de requerimientos</t>
   </si>
   <si>
-    <t>2026-04-30</t>
-  </si>
-  <si>
     <t>Fase 2: diseño</t>
   </si>
   <si>
     <t>Diseño de interfaz de usuario</t>
   </si>
   <si>
-    <t>2026-05-01</t>
-  </si>
-  <si>
-    <t>2026-05-07</t>
-  </si>
-  <si>
     <t>Prototipos</t>
   </si>
   <si>
-    <t>2026-05-04</t>
-  </si>
-  <si>
-    <t>2026-05-10</t>
-  </si>
-  <si>
     <t>Establecer lenguaje/programación</t>
   </si>
   <si>
-    <t>2026-05-06</t>
-  </si>
-  <si>
-    <t>2026-05-11</t>
-  </si>
-  <si>
     <t>Documentación del diseño</t>
   </si>
   <si>
-    <t>2026-05-09</t>
-  </si>
-  <si>
-    <t>2026-05-14</t>
-  </si>
-  <si>
     <t>Fase 3: desarrollo</t>
   </si>
   <si>
     <t>Crear código fuente</t>
   </si>
   <si>
-    <t>2026-05-12</t>
-  </si>
-  <si>
-    <t>2026-05-28</t>
-  </si>
-  <si>
     <t>Ejecución e integración del código</t>
   </si>
   <si>
-    <t>2026-05-18</t>
-  </si>
-  <si>
-    <t>2026-05-31</t>
-  </si>
-  <si>
     <t>Fase 4: pruebas</t>
   </si>
   <si>
     <t>Pruebas unitarias</t>
   </si>
   <si>
-    <t>2026-06-01</t>
-  </si>
-  <si>
-    <t>2026-06-06</t>
-  </si>
-  <si>
     <t>Pruebas de integración</t>
   </si>
   <si>
-    <t>2026-06-03</t>
-  </si>
-  <si>
-    <t>2026-06-08</t>
-  </si>
-  <si>
     <t>Pruebas de seguridad</t>
   </si>
   <si>
-    <t>2026-06-04</t>
-  </si>
-  <si>
-    <t>2026-06-10</t>
-  </si>
-  <si>
     <t>Pruebas de rendimiento</t>
   </si>
   <si>
-    <t>2026-06-15</t>
-  </si>
-  <si>
     <t>En curso</t>
   </si>
   <si>
     <t>Pruebas de compatibilidad</t>
   </si>
   <si>
-    <t>2026-06-16</t>
-  </si>
-  <si>
     <t>Pruebas de almacenamiento</t>
   </si>
   <si>
-    <t>2026-06-12</t>
-  </si>
-  <si>
-    <t>2026-06-18</t>
-  </si>
-  <si>
     <t>Planeado</t>
   </si>
   <si>
     <t>Documentación de pruebas</t>
   </si>
   <si>
-    <t>2026-06-14</t>
-  </si>
-  <si>
-    <t>2026-06-21</t>
-  </si>
-  <si>
     <t>Fase 5: entrega</t>
   </si>
   <si>
     <t>Copias de seguridad</t>
   </si>
   <si>
-    <t>2026-06-22</t>
-  </si>
-  <si>
     <t>Prueba de validación</t>
   </si>
   <si>
-    <t>2026-06-20</t>
-  </si>
-  <si>
-    <t>2026-06-24</t>
-  </si>
-  <si>
     <t>Capacitación del personal</t>
   </si>
   <si>
-    <t>2026-06-27</t>
-  </si>
-  <si>
     <t>Entrega del software y documentación</t>
-  </si>
-  <si>
-    <t>2026-06-30</t>
   </si>
   <si>
     <t>Leyenda</t>
@@ -1400,7 +1301,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="23">
+  <borders count="31">
     <border>
       <left/>
       <right/>
@@ -1682,11 +1583,119 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB7B7B7"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FFB7B7B7"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB7B7B7"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB7B7B7"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB7B7B7"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB7B7B7"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB7B7B7"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB7B7B7"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFB7B7B7"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="2"/>
+      </left>
+      <right style="thin">
+        <color theme="2"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color theme="2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="2" tint="-9.9978637043366805E-2"/>
+      </left>
+      <right style="thin">
+        <color theme="2" tint="-9.9978637043366805E-2"/>
+      </right>
+      <top style="thin">
+        <color theme="2" tint="-9.9978637043366805E-2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB7B7B7"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="2" tint="-9.9978637043366805E-2"/>
+      </left>
+      <right style="thin">
+        <color theme="2" tint="-9.9978637043366805E-2"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB7B7B7"/>
+      </top>
+      <bottom style="thin">
+        <color theme="2" tint="-9.9978637043366805E-2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FFB7B7B7"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB7B7B7"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="2" tint="-9.9978637043366805E-2"/>
+      </left>
+      <right style="thin">
+        <color theme="2" tint="-9.9978637043366805E-2"/>
+      </right>
+      <top style="thin">
+        <color theme="2" tint="-9.9978637043366805E-2"/>
+      </top>
+      <bottom style="thin">
+        <color theme="2" tint="-9.9978637043366805E-2"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="87">
+  <cellXfs count="99">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1778,24 +1787,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="6" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="21" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="22" fillId="7" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="21" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="23" fillId="8" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="21" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="19" fillId="6" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="6" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1814,6 +1810,46 @@
     </xf>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="21" fillId="6" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="7" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="8" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="6" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="6" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="30" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="30" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="30" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="26" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1845,7 +1881,6 @@
     <xf numFmtId="0" fontId="19" fillId="6" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1"/>
@@ -9274,417 +9309,417 @@
     <col min="2" max="2" width="40.140625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="54.28515625" customWidth="1"/>
     <col min="6" max="6" width="17.28515625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="7.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="2:8" ht="15"/>
     <row r="2" spans="2:8" ht="18.75">
-      <c r="B2" s="64" t="s">
+      <c r="B2" s="59" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="3" spans="2:8" ht="15.75">
-      <c r="B3" s="65" t="s">
+      <c r="B3" s="60" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="4" spans="2:8" ht="15">
-      <c r="B4" s="66" t="s">
+      <c r="B4" s="61" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="5" spans="2:8" ht="15">
-      <c r="B5" s="67" t="s">
+      <c r="B5" s="62" t="s">
         <v>3</v>
       </c>
-      <c r="C5" s="67" t="s">
+      <c r="C5" s="62" t="s">
         <v>4</v>
       </c>
-      <c r="F5" s="67" t="s">
+      <c r="F5" s="62" t="s">
         <v>5</v>
       </c>
-      <c r="G5" s="67" t="s">
+      <c r="G5" s="62" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="6" spans="2:8" ht="72.75">
-      <c r="B6" s="68" t="s">
+      <c r="B6" s="63" t="s">
         <v>7</v>
       </c>
-      <c r="C6" s="68" t="s">
+      <c r="C6" s="63" t="s">
         <v>8</v>
       </c>
-      <c r="F6" s="68" t="s">
+      <c r="F6" s="63" t="s">
         <v>9</v>
       </c>
-      <c r="G6" s="68" cm="1">
+      <c r="G6" s="63" cm="1">
         <f t="array" ref="G6">Tabla3235[[total de requerimintos ]]+Tabla32[[total de requerimintos ]]+Tabla323[[total de requerimintos ]]+Tabla3236[[total de requerimintos ]]+Tabla32367[[total de requerimintos ]]+Tabla323678[[total de requerimintos ]]</f>
         <v>158</v>
       </c>
     </row>
     <row r="7" spans="2:8" ht="57.75">
-      <c r="B7" s="68" t="s">
+      <c r="B7" s="63" t="s">
         <v>10</v>
       </c>
-      <c r="C7" s="68" t="s">
+      <c r="C7" s="63" t="s">
         <v>11</v>
       </c>
-      <c r="F7" s="68" t="s">
+      <c r="F7" s="63" t="s">
         <v>12</v>
       </c>
-      <c r="G7" s="68" cm="1">
+      <c r="G7" s="63" cm="1">
         <f t="array" ref="G7">Tabla3235[[Requeriminetos cumplidos ]]+Tabla32[[Requeriminetos cumplidos ]]+Tabla323[[Requeriminetos cumplidos ]]+Tabla3236[[Requeriminetos cumplidos ]]+Tabla32367[[Requeriminetos cumplidos ]]+Tabla323678[[Requeriminetos cumplidos ]]</f>
         <v>129</v>
       </c>
     </row>
     <row r="8" spans="2:8" ht="43.5">
-      <c r="B8" s="68" t="s">
+      <c r="B8" s="63" t="s">
         <v>13</v>
       </c>
-      <c r="C8" s="68" t="s">
+      <c r="C8" s="63" t="s">
         <v>14</v>
       </c>
-      <c r="F8" s="68" t="s">
+      <c r="F8" s="63" t="s">
         <v>15</v>
       </c>
-      <c r="G8" s="68" cm="1">
+      <c r="G8" s="63" cm="1">
         <f t="array" ref="G8">Tabla3235[Requeriminetos parcial]+Tabla32[Requeriminetos parcial]+Tabla323[Requeriminetos parcial]+Tabla3236[Requeriminetos parcial]+Tabla32367[Requeriminetos parcial]+Tabla323678[Requeriminetos parcial]</f>
         <v>25</v>
       </c>
     </row>
     <row r="9" spans="2:8" ht="43.5">
-      <c r="B9" s="68" t="s">
+      <c r="B9" s="63" t="s">
         <v>16</v>
       </c>
-      <c r="C9" s="68" t="s">
+      <c r="C9" s="63" t="s">
         <v>17</v>
       </c>
-      <c r="F9" s="68" t="s">
+      <c r="F9" s="63" t="s">
         <v>18</v>
       </c>
-      <c r="G9" s="68" cm="1">
+      <c r="G9" s="63" cm="1">
         <f t="array" ref="G9">Tabla3235[Requeriminetos no]+Tabla32[Requeriminetos no]+Tabla323[Requeriminetos no]+Tabla3236[Requeriminetos no]+Tabla32367[Requeriminetos no]+Tabla323678[Requeriminetos no]</f>
         <v>4</v>
       </c>
     </row>
     <row r="10" spans="2:8" ht="43.5">
-      <c r="B10" s="68" t="s">
+      <c r="B10" s="63" t="s">
         <v>19</v>
       </c>
-      <c r="C10" s="68" t="s">
+      <c r="C10" s="63" t="s">
         <v>20</v>
       </c>
-      <c r="F10" s="68" t="s">
+      <c r="F10" s="63" t="s">
         <v>21</v>
       </c>
-      <c r="G10" s="69">
+      <c r="G10" s="64">
         <f>(G7/G6)</f>
         <v>0.81645569620253167</v>
       </c>
-      <c r="H10" s="69"/>
+      <c r="H10" s="64"/>
     </row>
     <row r="11" spans="2:8" ht="57.75">
-      <c r="B11" s="68" t="s">
+      <c r="B11" s="63" t="s">
         <v>22</v>
       </c>
-      <c r="C11" s="68" t="s">
+      <c r="C11" s="63" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="12" spans="2:8" ht="43.5">
-      <c r="B12" s="68" t="s">
+      <c r="B12" s="63" t="s">
         <v>24</v>
       </c>
-      <c r="C12" s="68" t="s">
+      <c r="C12" s="63" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="13" spans="2:8" ht="57.75">
-      <c r="B13" s="68" t="s">
+      <c r="B13" s="63" t="s">
         <v>26</v>
       </c>
-      <c r="C13" s="68" t="s">
+      <c r="C13" s="63" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="14" spans="2:8" ht="43.5">
-      <c r="B14" s="68" t="s">
+      <c r="B14" s="63" t="s">
         <v>28</v>
       </c>
-      <c r="C14" s="68" t="s">
+      <c r="C14" s="63" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="15" spans="2:8" ht="43.5">
-      <c r="B15" s="68" t="s">
+      <c r="B15" s="63" t="s">
         <v>30</v>
       </c>
-      <c r="C15" s="68" t="s">
+      <c r="C15" s="63" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="16" spans="2:8" ht="29.25">
-      <c r="B16" s="68" t="s">
+      <c r="B16" s="63" t="s">
         <v>32</v>
       </c>
-      <c r="C16" s="68" t="s">
+      <c r="C16" s="63" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="17" spans="2:3" ht="43.5">
-      <c r="B17" s="68" t="s">
+      <c r="B17" s="63" t="s">
         <v>34</v>
       </c>
-      <c r="C17" s="68" t="s">
+      <c r="C17" s="63" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="18" spans="2:3" ht="43.5">
-      <c r="B18" s="68" t="s">
+      <c r="B18" s="63" t="s">
         <v>36</v>
       </c>
-      <c r="C18" s="68" t="s">
+      <c r="C18" s="63" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="19" spans="2:3" ht="43.5">
-      <c r="B19" s="68" t="s">
+      <c r="B19" s="63" t="s">
         <v>38</v>
       </c>
-      <c r="C19" s="68" t="s">
+      <c r="C19" s="63" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="20" spans="2:3" ht="43.5">
-      <c r="B20" s="68" t="s">
+      <c r="B20" s="63" t="s">
         <v>40</v>
       </c>
-      <c r="C20" s="68" t="s">
+      <c r="C20" s="63" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="21" spans="2:3" ht="43.5">
-      <c r="B21" s="68" t="s">
+      <c r="B21" s="63" t="s">
         <v>42</v>
       </c>
-      <c r="C21" s="68" t="s">
+      <c r="C21" s="63" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="22" spans="2:3" ht="43.5">
-      <c r="B22" s="68" t="s">
+      <c r="B22" s="63" t="s">
         <v>44</v>
       </c>
-      <c r="C22" s="68" t="s">
+      <c r="C22" s="63" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="23" spans="2:3" ht="43.5">
-      <c r="B23" s="68" t="s">
+      <c r="B23" s="63" t="s">
         <v>46</v>
       </c>
-      <c r="C23" s="68" t="s">
+      <c r="C23" s="63" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="24" spans="2:3" ht="43.5">
-      <c r="B24" s="68" t="s">
+      <c r="B24" s="63" t="s">
         <v>48</v>
       </c>
-      <c r="C24" s="68" t="s">
+      <c r="C24" s="63" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="25" spans="2:3" ht="43.5">
-      <c r="B25" s="68" t="s">
+      <c r="B25" s="63" t="s">
         <v>50</v>
       </c>
-      <c r="C25" s="68" t="s">
+      <c r="C25" s="63" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="26" spans="2:3" ht="43.5">
-      <c r="B26" s="68" t="s">
+      <c r="B26" s="63" t="s">
         <v>52</v>
       </c>
-      <c r="C26" s="68" t="s">
+      <c r="C26" s="63" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="27" spans="2:3" ht="43.5">
-      <c r="B27" s="68" t="s">
+      <c r="B27" s="63" t="s">
         <v>54</v>
       </c>
-      <c r="C27" s="68" t="s">
+      <c r="C27" s="63" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="28" spans="2:3" ht="15"/>
     <row r="29" spans="2:3" ht="15">
-      <c r="B29" s="67" t="s">
+      <c r="B29" s="62" t="s">
         <v>56</v>
       </c>
-      <c r="C29" s="67" t="s">
+      <c r="C29" s="62" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="30" spans="2:3" ht="15">
-      <c r="B30" s="68" t="s">
+      <c r="B30" s="63" t="s">
         <v>58</v>
       </c>
-      <c r="C30" s="68" t="s">
+      <c r="C30" s="63" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="31" spans="2:3" ht="15">
-      <c r="B31" s="68" t="s">
+      <c r="B31" s="63" t="s">
         <v>60</v>
       </c>
-      <c r="C31" s="68" t="s">
+      <c r="C31" s="63" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="32" spans="2:3" ht="15">
-      <c r="B32" s="68" t="s">
+      <c r="B32" s="63" t="s">
         <v>62</v>
       </c>
-      <c r="C32" s="68" t="s">
+      <c r="C32" s="63" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="33" spans="2:3" ht="15">
-      <c r="B33" s="68" t="s">
+      <c r="B33" s="63" t="s">
         <v>64</v>
       </c>
-      <c r="C33" s="68" t="s">
+      <c r="C33" s="63" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="34" spans="2:3" ht="15">
-      <c r="B34" s="68" t="s">
+      <c r="B34" s="63" t="s">
         <v>66</v>
       </c>
-      <c r="C34" s="68" t="s">
+      <c r="C34" s="63" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="35" spans="2:3" ht="15">
-      <c r="B35" s="68" t="s">
+      <c r="B35" s="63" t="s">
         <v>68</v>
       </c>
-      <c r="C35" s="68" t="s">
+      <c r="C35" s="63" t="s">
         <v>69</v>
       </c>
     </row>
     <row r="36" spans="2:3" ht="29.25">
-      <c r="B36" s="68" t="s">
+      <c r="B36" s="63" t="s">
         <v>70</v>
       </c>
-      <c r="C36" s="68" t="s">
+      <c r="C36" s="63" t="s">
         <v>71</v>
       </c>
     </row>
     <row r="37" spans="2:3" ht="15">
-      <c r="B37" s="68" t="s">
+      <c r="B37" s="63" t="s">
         <v>72</v>
       </c>
-      <c r="C37" s="68" t="s">
+      <c r="C37" s="63" t="s">
         <v>73</v>
       </c>
     </row>
     <row r="38" spans="2:3" ht="29.25">
-      <c r="B38" s="68" t="s">
+      <c r="B38" s="63" t="s">
         <v>74</v>
       </c>
-      <c r="C38" s="68" t="s">
+      <c r="C38" s="63" t="s">
         <v>75</v>
       </c>
     </row>
     <row r="39" spans="2:3" ht="15">
-      <c r="B39" s="68" t="s">
+      <c r="B39" s="63" t="s">
         <v>76</v>
       </c>
-      <c r="C39" s="68" t="s">
+      <c r="C39" s="63" t="s">
         <v>77</v>
       </c>
     </row>
     <row r="40" spans="2:3" ht="29.25">
-      <c r="B40" s="68" t="s">
+      <c r="B40" s="63" t="s">
         <v>78</v>
       </c>
-      <c r="C40" s="68" t="s">
+      <c r="C40" s="63" t="s">
         <v>79</v>
       </c>
     </row>
     <row r="41" spans="2:3" ht="29.25">
-      <c r="B41" s="68" t="s">
+      <c r="B41" s="63" t="s">
         <v>80</v>
       </c>
-      <c r="C41" s="68" t="s">
+      <c r="C41" s="63" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="42" spans="2:3" ht="15">
-      <c r="B42" s="68" t="s">
+      <c r="B42" s="63" t="s">
         <v>82</v>
       </c>
-      <c r="C42" s="68" t="s">
+      <c r="C42" s="63" t="s">
         <v>83</v>
       </c>
     </row>
     <row r="43" spans="2:3" ht="15">
-      <c r="B43" s="68" t="s">
+      <c r="B43" s="63" t="s">
         <v>84</v>
       </c>
-      <c r="C43" s="68" t="s">
+      <c r="C43" s="63" t="s">
         <v>85</v>
       </c>
     </row>
     <row r="44" spans="2:3" ht="15">
-      <c r="B44" s="68" t="s">
+      <c r="B44" s="63" t="s">
         <v>86</v>
       </c>
-      <c r="C44" s="68" t="s">
+      <c r="C44" s="63" t="s">
         <v>87</v>
       </c>
     </row>
     <row r="45" spans="2:3" ht="15">
-      <c r="B45" s="68" t="s">
+      <c r="B45" s="63" t="s">
         <v>88</v>
       </c>
-      <c r="C45" s="68" t="s">
+      <c r="C45" s="63" t="s">
         <v>89</v>
       </c>
     </row>
     <row r="46" spans="2:3" ht="15">
-      <c r="B46" s="68" t="s">
+      <c r="B46" s="63" t="s">
         <v>90</v>
       </c>
-      <c r="C46" s="68" t="s">
+      <c r="C46" s="63" t="s">
         <v>91</v>
       </c>
     </row>
     <row r="47" spans="2:3" ht="15">
-      <c r="B47" s="68" t="s">
+      <c r="B47" s="63" t="s">
         <v>92</v>
       </c>
-      <c r="C47" s="68" t="s">
+      <c r="C47" s="63" t="s">
         <v>93</v>
       </c>
     </row>
     <row r="48" spans="2:3" ht="15">
-      <c r="B48" s="68" t="s">
+      <c r="B48" s="63" t="s">
         <v>94</v>
       </c>
-      <c r="C48" s="68" t="s">
+      <c r="C48" s="63" t="s">
         <v>95</v>
       </c>
     </row>
     <row r="49" spans="2:3" ht="15">
-      <c r="B49" s="68" t="s">
+      <c r="B49" s="63" t="s">
         <v>96</v>
       </c>
-      <c r="C49" s="68" t="s">
+      <c r="C49" s="63" t="s">
         <v>97</v>
       </c>
     </row>
@@ -9711,15 +9746,15 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:13" ht="47.45" customHeight="1">
-      <c r="B2" s="73" t="s">
+      <c r="B2" s="86" t="s">
         <v>98</v>
       </c>
-      <c r="C2" s="81"/>
-      <c r="D2" s="81"/>
-      <c r="E2" s="81"/>
-      <c r="F2" s="81"/>
-      <c r="G2" s="81"/>
-      <c r="H2" s="81"/>
+      <c r="C2" s="93"/>
+      <c r="D2" s="93"/>
+      <c r="E2" s="93"/>
+      <c r="F2" s="93"/>
+      <c r="G2" s="93"/>
+      <c r="H2" s="93"/>
     </row>
     <row r="3" spans="2:13">
       <c r="B3" s="1"/>
@@ -9750,30 +9785,30 @@
       </c>
     </row>
     <row r="7" spans="2:13" ht="15.6" customHeight="1">
-      <c r="B7" s="71" t="s">
+      <c r="B7" s="84" t="s">
         <v>105</v>
       </c>
-      <c r="C7" s="81"/>
+      <c r="C7" s="93"/>
     </row>
     <row r="8" spans="2:13" ht="15.6" customHeight="1">
       <c r="B8" s="4"/>
       <c r="C8" s="4"/>
     </row>
     <row r="9" spans="2:13" ht="15">
-      <c r="E9" s="70" t="s">
+      <c r="E9" s="83" t="s">
         <v>106</v>
       </c>
-      <c r="F9" s="82"/>
-      <c r="G9" s="83"/>
-      <c r="H9" s="70" t="s">
+      <c r="F9" s="94"/>
+      <c r="G9" s="95"/>
+      <c r="H9" s="83" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="10" spans="2:13" ht="18" customHeight="1">
-      <c r="B10" s="72" t="s">
+      <c r="B10" s="85" t="s">
         <v>108</v>
       </c>
-      <c r="C10" s="84"/>
+      <c r="C10" s="96"/>
       <c r="D10" s="5"/>
       <c r="E10" s="6" t="s">
         <v>99</v>
@@ -9784,7 +9819,7 @@
       <c r="G10" s="7" t="s">
         <v>101</v>
       </c>
-      <c r="H10" s="85"/>
+      <c r="H10" s="97"/>
       <c r="I10" s="8"/>
     </row>
     <row r="11" spans="2:13">
@@ -10155,16 +10190,16 @@
       <c r="B35" s="13">
         <v>24</v>
       </c>
-      <c r="C35" s="60" t="s">
+      <c r="C35" s="55" t="s">
         <v>138</v>
       </c>
       <c r="D35" s="15"/>
       <c r="E35" s="45" t="s">
         <v>111</v>
       </c>
-      <c r="F35" s="63"/>
-      <c r="G35" s="63"/>
-      <c r="H35" s="63"/>
+      <c r="F35" s="58"/>
+      <c r="G35" s="58"/>
+      <c r="H35" s="58"/>
     </row>
     <row r="36" spans="2:8" ht="28.5">
       <c r="B36" s="13">
@@ -10316,15 +10351,15 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:13" ht="47.45" customHeight="1">
-      <c r="B2" s="77" t="s">
+      <c r="B2" s="90" t="s">
         <v>98</v>
       </c>
-      <c r="C2" s="86"/>
-      <c r="D2" s="86"/>
-      <c r="E2" s="86"/>
-      <c r="F2" s="86"/>
-      <c r="G2" s="86"/>
-      <c r="H2" s="86"/>
+      <c r="C2" s="98"/>
+      <c r="D2" s="98"/>
+      <c r="E2" s="98"/>
+      <c r="F2" s="98"/>
+      <c r="G2" s="98"/>
+      <c r="H2" s="98"/>
     </row>
     <row r="3" spans="2:13">
       <c r="B3" s="19"/>
@@ -10355,30 +10390,30 @@
       </c>
     </row>
     <row r="7" spans="2:13" ht="15.6" customHeight="1">
-      <c r="B7" s="75" t="s">
+      <c r="B7" s="88" t="s">
         <v>105</v>
       </c>
-      <c r="C7" s="86"/>
+      <c r="C7" s="98"/>
     </row>
     <row r="8" spans="2:13" ht="15.6" customHeight="1">
       <c r="B8" s="22"/>
       <c r="C8" s="22"/>
     </row>
     <row r="9" spans="2:13">
-      <c r="E9" s="74" t="s">
+      <c r="E9" s="87" t="s">
         <v>106</v>
       </c>
-      <c r="F9" s="82"/>
-      <c r="G9" s="83"/>
-      <c r="H9" s="74" t="s">
+      <c r="F9" s="94"/>
+      <c r="G9" s="95"/>
+      <c r="H9" s="87" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="10" spans="2:13" ht="17.45" customHeight="1">
-      <c r="B10" s="76" t="s">
+      <c r="B10" s="89" t="s">
         <v>147</v>
       </c>
-      <c r="C10" s="84"/>
+      <c r="C10" s="96"/>
       <c r="D10" s="23"/>
       <c r="E10" s="24" t="s">
         <v>99</v>
@@ -10389,7 +10424,7 @@
       <c r="G10" s="25" t="s">
         <v>101</v>
       </c>
-      <c r="H10" s="85"/>
+      <c r="H10" s="97"/>
       <c r="I10" s="26"/>
     </row>
     <row r="11" spans="2:13">
@@ -10653,7 +10688,7 @@
       <c r="B28" s="34">
         <v>17</v>
       </c>
-      <c r="C28" s="60" t="s">
+      <c r="C28" s="55" t="s">
         <v>164</v>
       </c>
       <c r="E28" s="33" t="s">
@@ -10663,75 +10698,75 @@
       <c r="G28" s="33"/>
       <c r="H28" s="33"/>
     </row>
-    <row r="29" spans="2:8" s="61" customFormat="1" ht="28.5">
+    <row r="29" spans="2:8" s="56" customFormat="1" ht="28.5">
       <c r="B29" s="30">
         <v>18</v>
       </c>
       <c r="C29" s="38" t="s">
         <v>165</v>
       </c>
-      <c r="E29" s="62" t="s">
-        <v>111</v>
-      </c>
-      <c r="F29" s="62"/>
-      <c r="G29" s="62"/>
-      <c r="H29" s="62"/>
-    </row>
-    <row r="30" spans="2:8" s="61" customFormat="1" ht="28.5">
+      <c r="E29" s="57" t="s">
+        <v>111</v>
+      </c>
+      <c r="F29" s="57"/>
+      <c r="G29" s="57"/>
+      <c r="H29" s="57"/>
+    </row>
+    <row r="30" spans="2:8" s="56" customFormat="1" ht="28.5">
       <c r="B30" s="30">
         <v>19</v>
       </c>
       <c r="C30" s="38" t="s">
         <v>166</v>
       </c>
-      <c r="E30" s="62" t="s">
-        <v>111</v>
-      </c>
-      <c r="F30" s="62"/>
-      <c r="G30" s="62"/>
-      <c r="H30" s="62"/>
-    </row>
-    <row r="31" spans="2:8" s="61" customFormat="1" ht="14.25">
+      <c r="E30" s="57" t="s">
+        <v>111</v>
+      </c>
+      <c r="F30" s="57"/>
+      <c r="G30" s="57"/>
+      <c r="H30" s="57"/>
+    </row>
+    <row r="31" spans="2:8" s="56" customFormat="1" ht="14.25">
       <c r="B31" s="30">
         <v>20</v>
       </c>
       <c r="C31" s="38" t="s">
         <v>167</v>
       </c>
-      <c r="E31" s="62" t="s">
-        <v>111</v>
-      </c>
-      <c r="F31" s="62"/>
-      <c r="G31" s="62"/>
-      <c r="H31" s="62"/>
-    </row>
-    <row r="32" spans="2:8" s="61" customFormat="1" ht="28.5">
+      <c r="E31" s="57" t="s">
+        <v>111</v>
+      </c>
+      <c r="F31" s="57"/>
+      <c r="G31" s="57"/>
+      <c r="H31" s="57"/>
+    </row>
+    <row r="32" spans="2:8" s="56" customFormat="1" ht="28.5">
       <c r="B32" s="34">
         <v>21</v>
       </c>
       <c r="C32" s="38" t="s">
         <v>168</v>
       </c>
-      <c r="E32" s="62" t="s">
-        <v>111</v>
-      </c>
-      <c r="F32" s="62"/>
-      <c r="G32" s="62"/>
-      <c r="H32" s="62"/>
-    </row>
-    <row r="33" spans="2:8" s="61" customFormat="1" ht="28.5">
+      <c r="E32" s="57" t="s">
+        <v>111</v>
+      </c>
+      <c r="F32" s="57"/>
+      <c r="G32" s="57"/>
+      <c r="H32" s="57"/>
+    </row>
+    <row r="33" spans="2:8" s="56" customFormat="1" ht="28.5">
       <c r="B33" s="30">
         <v>22</v>
       </c>
       <c r="C33" s="38" t="s">
         <v>169</v>
       </c>
-      <c r="E33" s="62" t="s">
-        <v>111</v>
-      </c>
-      <c r="F33" s="62"/>
-      <c r="G33" s="62"/>
-      <c r="H33" s="62"/>
+      <c r="E33" s="57" t="s">
+        <v>111</v>
+      </c>
+      <c r="F33" s="57"/>
+      <c r="G33" s="57"/>
+      <c r="H33" s="57"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -10768,15 +10803,15 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:13" ht="47.45" customHeight="1">
-      <c r="B2" s="77" t="s">
+      <c r="B2" s="90" t="s">
         <v>98</v>
       </c>
-      <c r="C2" s="86"/>
-      <c r="D2" s="86"/>
-      <c r="E2" s="86"/>
-      <c r="F2" s="86"/>
-      <c r="G2" s="86"/>
-      <c r="H2" s="86"/>
+      <c r="C2" s="98"/>
+      <c r="D2" s="98"/>
+      <c r="E2" s="98"/>
+      <c r="F2" s="98"/>
+      <c r="G2" s="98"/>
+      <c r="H2" s="98"/>
     </row>
     <row r="3" spans="2:13">
       <c r="B3" s="19"/>
@@ -10807,30 +10842,30 @@
       </c>
     </row>
     <row r="7" spans="2:13" ht="15.6" customHeight="1">
-      <c r="B7" s="75" t="s">
+      <c r="B7" s="88" t="s">
         <v>105</v>
       </c>
-      <c r="C7" s="86"/>
+      <c r="C7" s="98"/>
     </row>
     <row r="8" spans="2:13" ht="15.6" customHeight="1">
       <c r="B8" s="22"/>
       <c r="C8" s="22"/>
     </row>
     <row r="9" spans="2:13">
-      <c r="E9" s="74" t="s">
+      <c r="E9" s="87" t="s">
         <v>106</v>
       </c>
-      <c r="F9" s="82"/>
-      <c r="G9" s="83"/>
-      <c r="H9" s="74" t="s">
+      <c r="F9" s="94"/>
+      <c r="G9" s="95"/>
+      <c r="H9" s="87" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="10" spans="2:13" ht="17.45" customHeight="1">
-      <c r="B10" s="76" t="s">
+      <c r="B10" s="89" t="s">
         <v>170</v>
       </c>
-      <c r="C10" s="84"/>
+      <c r="C10" s="96"/>
       <c r="D10" s="23"/>
       <c r="E10" s="24" t="s">
         <v>99</v>
@@ -10841,7 +10876,7 @@
       <c r="G10" s="25" t="s">
         <v>101</v>
       </c>
-      <c r="H10" s="85"/>
+      <c r="H10" s="97"/>
       <c r="I10" s="26"/>
     </row>
     <row r="11" spans="2:13">
@@ -11263,7 +11298,7 @@
       <c r="B39" s="30">
         <v>28</v>
       </c>
-      <c r="C39" s="60" t="s">
+      <c r="C39" s="55" t="s">
         <v>200</v>
       </c>
       <c r="E39" s="33" t="s">
@@ -11409,15 +11444,15 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:13" ht="47.45" customHeight="1">
-      <c r="B2" s="77" t="s">
+      <c r="B2" s="90" t="s">
         <v>98</v>
       </c>
-      <c r="C2" s="86"/>
-      <c r="D2" s="86"/>
-      <c r="E2" s="86"/>
-      <c r="F2" s="86"/>
-      <c r="G2" s="86"/>
-      <c r="H2" s="86"/>
+      <c r="C2" s="98"/>
+      <c r="D2" s="98"/>
+      <c r="E2" s="98"/>
+      <c r="F2" s="98"/>
+      <c r="G2" s="98"/>
+      <c r="H2" s="98"/>
     </row>
     <row r="3" spans="2:13">
       <c r="B3" s="19"/>
@@ -11448,30 +11483,30 @@
       </c>
     </row>
     <row r="7" spans="2:13" ht="15.6" customHeight="1">
-      <c r="B7" s="75" t="s">
+      <c r="B7" s="88" t="s">
         <v>105</v>
       </c>
-      <c r="C7" s="86"/>
+      <c r="C7" s="98"/>
     </row>
     <row r="8" spans="2:13" ht="15.6" customHeight="1">
       <c r="B8" s="22"/>
       <c r="C8" s="22"/>
     </row>
     <row r="9" spans="2:13">
-      <c r="E9" s="74" t="s">
+      <c r="E9" s="87" t="s">
         <v>106</v>
       </c>
-      <c r="F9" s="82"/>
-      <c r="G9" s="83"/>
-      <c r="H9" s="74" t="s">
+      <c r="F9" s="94"/>
+      <c r="G9" s="95"/>
+      <c r="H9" s="87" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="10" spans="2:13" ht="17.45" customHeight="1">
-      <c r="B10" s="76" t="s">
+      <c r="B10" s="89" t="s">
         <v>209</v>
       </c>
-      <c r="C10" s="84"/>
+      <c r="C10" s="96"/>
       <c r="D10" s="23"/>
       <c r="E10" s="24" t="s">
         <v>99</v>
@@ -11482,7 +11517,7 @@
       <c r="G10" s="25" t="s">
         <v>101</v>
       </c>
-      <c r="H10" s="85"/>
+      <c r="H10" s="97"/>
       <c r="I10" s="26"/>
     </row>
     <row r="11" spans="2:13">
@@ -11842,7 +11877,7 @@
       <c r="B34" s="34">
         <v>23</v>
       </c>
-      <c r="C34" s="60" t="s">
+      <c r="C34" s="55" t="s">
         <v>238</v>
       </c>
       <c r="E34" s="33" t="s">
@@ -11917,15 +11952,15 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:13" ht="47.45" customHeight="1">
-      <c r="B2" s="77" t="s">
+      <c r="B2" s="90" t="s">
         <v>98</v>
       </c>
-      <c r="C2" s="86"/>
-      <c r="D2" s="86"/>
-      <c r="E2" s="86"/>
-      <c r="F2" s="86"/>
-      <c r="G2" s="86"/>
-      <c r="H2" s="86"/>
+      <c r="C2" s="98"/>
+      <c r="D2" s="98"/>
+      <c r="E2" s="98"/>
+      <c r="F2" s="98"/>
+      <c r="G2" s="98"/>
+      <c r="H2" s="98"/>
     </row>
     <row r="3" spans="2:13">
       <c r="B3" s="19"/>
@@ -11956,30 +11991,30 @@
       </c>
     </row>
     <row r="7" spans="2:13" ht="15.6" customHeight="1">
-      <c r="B7" s="75" t="s">
+      <c r="B7" s="88" t="s">
         <v>105</v>
       </c>
-      <c r="C7" s="86"/>
+      <c r="C7" s="98"/>
     </row>
     <row r="8" spans="2:13" ht="15.6" customHeight="1">
       <c r="B8" s="22"/>
       <c r="C8" s="22"/>
     </row>
     <row r="9" spans="2:13">
-      <c r="E9" s="74" t="s">
+      <c r="E9" s="87" t="s">
         <v>106</v>
       </c>
-      <c r="F9" s="82"/>
-      <c r="G9" s="83"/>
-      <c r="H9" s="74" t="s">
+      <c r="F9" s="94"/>
+      <c r="G9" s="95"/>
+      <c r="H9" s="87" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="10" spans="2:13" ht="17.45" customHeight="1">
-      <c r="B10" s="76" t="s">
+      <c r="B10" s="89" t="s">
         <v>242</v>
       </c>
-      <c r="C10" s="84"/>
+      <c r="C10" s="96"/>
       <c r="D10" s="23"/>
       <c r="E10" s="24" t="s">
         <v>99</v>
@@ -11990,7 +12025,7 @@
       <c r="G10" s="25" t="s">
         <v>101</v>
       </c>
-      <c r="H10" s="85"/>
+      <c r="H10" s="97"/>
       <c r="I10" s="26"/>
     </row>
     <row r="11" spans="2:13">
@@ -12310,7 +12345,7 @@
       <c r="B32" s="34">
         <v>21</v>
       </c>
-      <c r="C32" s="60" t="s">
+      <c r="C32" s="55" t="s">
         <v>263</v>
       </c>
       <c r="E32" s="33" t="s">
@@ -12419,15 +12454,15 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:13" ht="47.45" customHeight="1">
-      <c r="B2" s="77" t="s">
+      <c r="B2" s="90" t="s">
         <v>98</v>
       </c>
-      <c r="C2" s="86"/>
-      <c r="D2" s="86"/>
-      <c r="E2" s="86"/>
-      <c r="F2" s="86"/>
-      <c r="G2" s="86"/>
-      <c r="H2" s="86"/>
+      <c r="C2" s="98"/>
+      <c r="D2" s="98"/>
+      <c r="E2" s="98"/>
+      <c r="F2" s="98"/>
+      <c r="G2" s="98"/>
+      <c r="H2" s="98"/>
     </row>
     <row r="3" spans="2:13">
       <c r="B3" s="19"/>
@@ -12458,30 +12493,30 @@
       </c>
     </row>
     <row r="7" spans="2:13" ht="15.6" customHeight="1">
-      <c r="B7" s="75" t="s">
+      <c r="B7" s="88" t="s">
         <v>105</v>
       </c>
-      <c r="C7" s="86"/>
+      <c r="C7" s="98"/>
     </row>
     <row r="8" spans="2:13" ht="15.6" customHeight="1">
       <c r="B8" s="22"/>
       <c r="C8" s="22"/>
     </row>
     <row r="9" spans="2:13">
-      <c r="E9" s="74" t="s">
+      <c r="E9" s="87" t="s">
         <v>106</v>
       </c>
-      <c r="F9" s="82"/>
-      <c r="G9" s="83"/>
-      <c r="H9" s="74" t="s">
+      <c r="F9" s="94"/>
+      <c r="G9" s="95"/>
+      <c r="H9" s="87" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="10" spans="2:13" ht="17.45" customHeight="1">
-      <c r="B10" s="76" t="s">
+      <c r="B10" s="89" t="s">
         <v>268</v>
       </c>
-      <c r="C10" s="84"/>
+      <c r="C10" s="96"/>
       <c r="D10" s="23"/>
       <c r="E10" s="24" t="s">
         <v>99</v>
@@ -12492,7 +12527,7 @@
       <c r="G10" s="25" t="s">
         <v>101</v>
       </c>
-      <c r="H10" s="85"/>
+      <c r="H10" s="97"/>
       <c r="I10" s="26"/>
     </row>
     <row r="11" spans="2:13">
@@ -12756,7 +12791,7 @@
       <c r="B28" s="34">
         <v>17</v>
       </c>
-      <c r="C28" s="60" t="s">
+      <c r="C28" s="55" t="s">
         <v>285</v>
       </c>
       <c r="E28" s="33" t="s">
@@ -12835,35 +12870,36 @@
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
     <col min="2" max="2" width="52" customWidth="1"/>
-    <col min="3" max="4" width="12" customWidth="1"/>
+    <col min="3" max="3" width="12" customWidth="1"/>
+    <col min="4" max="4" width="16.85546875" customWidth="1"/>
     <col min="5" max="5" width="18" customWidth="1"/>
     <col min="6" max="6" width="12" customWidth="1"/>
     <col min="7" max="20" width="6" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:20" ht="24" customHeight="1">
-      <c r="A1" s="78" t="s">
+      <c r="A1" s="91" t="s">
         <v>288</v>
       </c>
-      <c r="B1" s="81"/>
-      <c r="C1" s="81"/>
-      <c r="D1" s="81"/>
-      <c r="E1" s="81"/>
-      <c r="F1" s="81"/>
-      <c r="G1" s="81"/>
-      <c r="H1" s="81"/>
-      <c r="I1" s="81"/>
-      <c r="J1" s="81"/>
-      <c r="K1" s="81"/>
-      <c r="L1" s="81"/>
-      <c r="M1" s="81"/>
-      <c r="N1" s="81"/>
-      <c r="O1" s="81"/>
-      <c r="P1" s="81"/>
-      <c r="Q1" s="81"/>
-      <c r="R1" s="81"/>
-      <c r="S1" s="81"/>
-      <c r="T1" s="81"/>
+      <c r="B1" s="93"/>
+      <c r="C1" s="93"/>
+      <c r="D1" s="93"/>
+      <c r="E1" s="93"/>
+      <c r="F1" s="93"/>
+      <c r="G1" s="93"/>
+      <c r="H1" s="93"/>
+      <c r="I1" s="93"/>
+      <c r="J1" s="93"/>
+      <c r="K1" s="93"/>
+      <c r="L1" s="93"/>
+      <c r="M1" s="93"/>
+      <c r="N1" s="93"/>
+      <c r="O1" s="93"/>
+      <c r="P1" s="93"/>
+      <c r="Q1" s="93"/>
+      <c r="R1" s="93"/>
+      <c r="S1" s="93"/>
+      <c r="T1" s="93"/>
     </row>
     <row r="2" spans="1:20">
       <c r="A2" s="48" t="s">
@@ -12880,78 +12916,78 @@
       </c>
     </row>
     <row r="3" spans="1:20">
-      <c r="G3" s="79" t="s">
+      <c r="G3" s="92" t="s">
         <v>293</v>
       </c>
-      <c r="H3" s="81"/>
-      <c r="I3" s="81"/>
-      <c r="J3" s="81"/>
-      <c r="K3" s="79" t="s">
+      <c r="H3" s="93"/>
+      <c r="I3" s="93"/>
+      <c r="J3" s="93"/>
+      <c r="K3" s="92" t="s">
         <v>294</v>
       </c>
-      <c r="L3" s="81"/>
-      <c r="M3" s="81"/>
-      <c r="N3" s="81"/>
-      <c r="O3" s="79" t="s">
+      <c r="L3" s="93"/>
+      <c r="M3" s="93"/>
+      <c r="N3" s="93"/>
+      <c r="O3" s="92" t="s">
         <v>295</v>
       </c>
-      <c r="P3" s="81"/>
-      <c r="Q3" s="81"/>
-      <c r="R3" s="81"/>
+      <c r="P3" s="93"/>
+      <c r="Q3" s="93"/>
+      <c r="R3" s="93"/>
     </row>
     <row r="4" spans="1:20" ht="29.25" customHeight="1">
-      <c r="A4" s="58" t="s">
+      <c r="A4" s="54" t="s">
         <v>296</v>
       </c>
-      <c r="B4" s="58" t="s">
+      <c r="B4" s="54" t="s">
         <v>297</v>
       </c>
-      <c r="C4" s="58" t="s">
+      <c r="C4" s="54" t="s">
         <v>298</v>
       </c>
-      <c r="D4" s="58" t="s">
+      <c r="D4" s="54" t="s">
         <v>299</v>
       </c>
-      <c r="E4" s="58" t="s">
+      <c r="E4" s="54" t="s">
         <v>300</v>
       </c>
-      <c r="F4" s="58" t="s">
+      <c r="F4" s="54" t="s">
         <v>301</v>
       </c>
-      <c r="G4" s="59" t="s">
+      <c r="G4" s="69" t="s">
         <v>302</v>
       </c>
-      <c r="H4" s="59" t="s">
+      <c r="H4" s="69" t="s">
         <v>303</v>
       </c>
-      <c r="I4" s="59" t="s">
+      <c r="I4" s="69" t="s">
         <v>304</v>
       </c>
-      <c r="J4" s="59" t="s">
+      <c r="J4" s="69" t="s">
         <v>305</v>
       </c>
-      <c r="K4" s="59" t="s">
+      <c r="K4" s="69" t="s">
         <v>302</v>
       </c>
-      <c r="L4" s="59" t="s">
+      <c r="L4" s="69" t="s">
         <v>303</v>
       </c>
-      <c r="M4" s="59" t="s">
+      <c r="M4" s="69" t="s">
         <v>304</v>
       </c>
-      <c r="N4" s="59" t="s">
+      <c r="N4" s="69" t="s">
         <v>305</v>
       </c>
-      <c r="O4" s="59" t="s">
+      <c r="O4" s="69" t="s">
         <v>302</v>
       </c>
-      <c r="P4" s="59" t="s">
+      <c r="P4" s="69" t="s">
         <v>303</v>
       </c>
-      <c r="Q4" s="59" t="s">
+      <c r="Q4" s="69" t="s">
         <v>304</v>
       </c>
-      <c r="R4" s="59" t="s">
+      <c r="R4" s="69" t="s">
         <v>305</v>
       </c>
     </row>
@@ -12962,588 +12998,627 @@
       <c r="B5" s="49" t="s">
         <v>307</v>
       </c>
-      <c r="C5" s="50" t="s">
+      <c r="C5" s="81">
+        <v>46141</v>
+      </c>
+      <c r="D5" s="81">
+        <v>46142</v>
+      </c>
+      <c r="E5" s="74">
+        <v>1</v>
+      </c>
+      <c r="F5" s="66" t="s">
         <v>308</v>
       </c>
-      <c r="D5" s="50" t="s">
-        <v>309</v>
-      </c>
-      <c r="E5" s="50">
-        <v>1</v>
-      </c>
-      <c r="F5" s="51" t="s">
-        <v>310</v>
-      </c>
-      <c r="G5" s="53"/>
-      <c r="H5" s="53"/>
-      <c r="I5" s="53"/>
-      <c r="J5" s="52"/>
-      <c r="K5" s="53"/>
-      <c r="L5" s="53"/>
-      <c r="M5" s="53"/>
-      <c r="N5" s="53"/>
-      <c r="O5" s="53"/>
-      <c r="P5" s="53"/>
-      <c r="Q5" s="53"/>
-      <c r="R5" s="53"/>
+      <c r="G5" s="76"/>
+      <c r="H5" s="76"/>
+      <c r="I5" s="76"/>
+      <c r="J5" s="77"/>
+      <c r="K5" s="76"/>
+      <c r="L5" s="76"/>
+      <c r="M5" s="76"/>
+      <c r="N5" s="76"/>
+      <c r="O5" s="76"/>
+      <c r="P5" s="76"/>
+      <c r="Q5" s="76"/>
+      <c r="R5" s="76"/>
     </row>
     <row r="6" spans="1:20" ht="24" customHeight="1">
       <c r="A6" s="49" t="s">
         <v>306</v>
       </c>
       <c r="B6" s="49" t="s">
-        <v>311</v>
-      </c>
-      <c r="C6" s="50" t="s">
         <v>309</v>
       </c>
-      <c r="D6" s="50" t="s">
-        <v>312</v>
-      </c>
-      <c r="E6" s="50">
+      <c r="C6" s="81">
+        <v>46141</v>
+      </c>
+      <c r="D6" s="82">
+        <v>46142</v>
+      </c>
+      <c r="E6" s="71">
         <v>1</v>
       </c>
-      <c r="F6" s="51" t="s">
-        <v>310</v>
-      </c>
-      <c r="G6" s="53"/>
-      <c r="H6" s="53"/>
-      <c r="I6" s="53"/>
-      <c r="J6" s="52"/>
-      <c r="K6" s="53"/>
-      <c r="L6" s="53"/>
-      <c r="M6" s="53"/>
-      <c r="N6" s="53"/>
-      <c r="O6" s="53"/>
-      <c r="P6" s="53"/>
-      <c r="Q6" s="53"/>
-      <c r="R6" s="53"/>
+      <c r="F6" s="73" t="s">
+        <v>308</v>
+      </c>
+      <c r="G6" s="76"/>
+      <c r="H6" s="76"/>
+      <c r="I6" s="76"/>
+      <c r="J6" s="77"/>
+      <c r="K6" s="76"/>
+      <c r="L6" s="76"/>
+      <c r="M6" s="76"/>
+      <c r="N6" s="76"/>
+      <c r="O6" s="76"/>
+      <c r="P6" s="76"/>
+      <c r="Q6" s="76"/>
+      <c r="R6" s="76"/>
     </row>
     <row r="7" spans="1:20" ht="24" customHeight="1">
       <c r="A7" s="49" t="s">
         <v>306</v>
       </c>
       <c r="B7" s="49" t="s">
-        <v>313</v>
-      </c>
-      <c r="C7" s="50" t="s">
-        <v>312</v>
-      </c>
-      <c r="D7" s="50" t="s">
-        <v>314</v>
-      </c>
-      <c r="E7" s="50">
+        <v>310</v>
+      </c>
+      <c r="C7" s="81">
+        <v>46141</v>
+      </c>
+      <c r="D7" s="82">
+        <v>46142</v>
+      </c>
+      <c r="E7" s="72">
         <v>1</v>
       </c>
-      <c r="F7" s="51" t="s">
-        <v>310</v>
-      </c>
-      <c r="G7" s="53"/>
-      <c r="H7" s="53"/>
-      <c r="I7" s="53"/>
-      <c r="J7" s="52"/>
-      <c r="K7" s="53"/>
-      <c r="L7" s="53"/>
-      <c r="M7" s="53"/>
-      <c r="N7" s="53"/>
-      <c r="O7" s="53"/>
-      <c r="P7" s="53"/>
-      <c r="Q7" s="53"/>
-      <c r="R7" s="53"/>
+      <c r="F7" s="73" t="s">
+        <v>308</v>
+      </c>
+      <c r="G7" s="76"/>
+      <c r="H7" s="76"/>
+      <c r="I7" s="76"/>
+      <c r="J7" s="77"/>
+      <c r="K7" s="76"/>
+      <c r="L7" s="76"/>
+      <c r="M7" s="76"/>
+      <c r="N7" s="76"/>
+      <c r="O7" s="76"/>
+      <c r="P7" s="76"/>
+      <c r="Q7" s="76"/>
+      <c r="R7" s="76"/>
     </row>
     <row r="8" spans="1:20" ht="24" customHeight="1">
       <c r="A8" s="49" t="s">
-        <v>315</v>
+        <v>311</v>
       </c>
       <c r="B8" s="49" t="s">
-        <v>316</v>
-      </c>
-      <c r="C8" s="50" t="s">
-        <v>317</v>
-      </c>
-      <c r="D8" s="50" t="s">
-        <v>318</v>
-      </c>
-      <c r="E8" s="50">
-        <v>1</v>
-      </c>
-      <c r="F8" s="51" t="s">
-        <v>310</v>
-      </c>
-      <c r="G8" s="53"/>
-      <c r="H8" s="53"/>
-      <c r="I8" s="53"/>
-      <c r="J8" s="53"/>
-      <c r="K8" s="52"/>
-      <c r="L8" s="53"/>
-      <c r="M8" s="53"/>
-      <c r="N8" s="53"/>
-      <c r="O8" s="53"/>
-      <c r="P8" s="53"/>
-      <c r="Q8" s="53"/>
-      <c r="R8" s="53"/>
+        <v>312</v>
+      </c>
+      <c r="C8" s="81">
+        <v>46141</v>
+      </c>
+      <c r="D8" s="81">
+        <v>46150</v>
+      </c>
+      <c r="E8" s="75">
+        <v>2</v>
+      </c>
+      <c r="F8" s="66" t="s">
+        <v>308</v>
+      </c>
+      <c r="G8" s="76"/>
+      <c r="H8" s="76"/>
+      <c r="I8" s="76"/>
+      <c r="J8" s="77"/>
+      <c r="K8" s="77"/>
+      <c r="L8" s="76"/>
+      <c r="M8" s="76"/>
+      <c r="N8" s="76"/>
+      <c r="O8" s="76"/>
+      <c r="P8" s="76"/>
+      <c r="Q8" s="76"/>
+      <c r="R8" s="76"/>
     </row>
     <row r="9" spans="1:20" ht="24" customHeight="1">
       <c r="A9" s="49" t="s">
-        <v>315</v>
+        <v>311</v>
       </c>
       <c r="B9" s="49" t="s">
-        <v>319</v>
-      </c>
-      <c r="C9" s="50" t="s">
-        <v>320</v>
-      </c>
-      <c r="D9" s="50" t="s">
-        <v>321</v>
+        <v>313</v>
+      </c>
+      <c r="C9" s="81">
+        <v>46141</v>
+      </c>
+      <c r="D9" s="81">
+        <v>46157</v>
       </c>
       <c r="E9" s="50">
-        <v>1</v>
-      </c>
-      <c r="F9" s="51" t="s">
-        <v>310</v>
-      </c>
-      <c r="G9" s="53"/>
-      <c r="H9" s="53"/>
-      <c r="I9" s="53"/>
-      <c r="J9" s="53"/>
-      <c r="K9" s="52"/>
-      <c r="L9" s="52"/>
-      <c r="M9" s="53"/>
-      <c r="N9" s="53"/>
-      <c r="O9" s="53"/>
-      <c r="P9" s="53"/>
-      <c r="Q9" s="53"/>
-      <c r="R9" s="53"/>
+        <v>3</v>
+      </c>
+      <c r="F9" s="66" t="s">
+        <v>308</v>
+      </c>
+      <c r="G9" s="76"/>
+      <c r="H9" s="76"/>
+      <c r="I9" s="76"/>
+      <c r="J9" s="77"/>
+      <c r="K9" s="77"/>
+      <c r="L9" s="77"/>
+      <c r="M9" s="76"/>
+      <c r="N9" s="76"/>
+      <c r="O9" s="76"/>
+      <c r="P9" s="76"/>
+      <c r="Q9" s="76"/>
+      <c r="R9" s="76"/>
     </row>
     <row r="10" spans="1:20" ht="24" customHeight="1">
       <c r="A10" s="49" t="s">
-        <v>315</v>
+        <v>311</v>
       </c>
       <c r="B10" s="49" t="s">
-        <v>322</v>
-      </c>
-      <c r="C10" s="50" t="s">
-        <v>323</v>
-      </c>
-      <c r="D10" s="50" t="s">
-        <v>324</v>
+        <v>314</v>
+      </c>
+      <c r="C10" s="81">
+        <v>46141</v>
+      </c>
+      <c r="D10" s="81">
+        <v>46169</v>
       </c>
       <c r="E10" s="50">
-        <v>1</v>
-      </c>
-      <c r="F10" s="51" t="s">
-        <v>310</v>
-      </c>
-      <c r="G10" s="53"/>
-      <c r="H10" s="53"/>
-      <c r="I10" s="52"/>
-      <c r="J10" s="52"/>
-      <c r="K10" s="53"/>
-      <c r="L10" s="53"/>
-      <c r="M10" s="53"/>
-      <c r="N10" s="53"/>
-      <c r="O10" s="53"/>
-      <c r="P10" s="53"/>
+        <v>4</v>
+      </c>
+      <c r="F10" s="66" t="s">
+        <v>308</v>
+      </c>
+      <c r="G10" s="76"/>
+      <c r="H10" s="76"/>
+      <c r="I10" s="76"/>
+      <c r="J10" s="77"/>
+      <c r="K10" s="77"/>
+      <c r="L10" s="77"/>
+      <c r="M10" s="77"/>
+      <c r="N10" s="76"/>
+      <c r="O10" s="76"/>
+      <c r="P10" s="76"/>
+      <c r="Q10" s="76"/>
+      <c r="R10" s="76"/>
     </row>
     <row r="11" spans="1:20" ht="24" customHeight="1">
       <c r="A11" s="49" t="s">
+        <v>311</v>
+      </c>
+      <c r="B11" s="49" t="s">
         <v>315</v>
       </c>
-      <c r="B11" s="49" t="s">
-        <v>325</v>
-      </c>
-      <c r="C11" s="50" t="s">
-        <v>326</v>
-      </c>
-      <c r="D11" s="50" t="s">
-        <v>327</v>
+      <c r="C11" s="81">
+        <v>46141</v>
+      </c>
+      <c r="D11" s="81">
+        <v>46169</v>
       </c>
       <c r="E11" s="50">
-        <v>1</v>
-      </c>
-      <c r="F11" s="51" t="s">
-        <v>310</v>
-      </c>
-      <c r="G11" s="53"/>
-      <c r="H11" s="53"/>
-      <c r="I11" s="52"/>
-      <c r="J11" s="52"/>
-      <c r="K11" s="53"/>
-      <c r="L11" s="53"/>
-      <c r="M11" s="53"/>
-      <c r="N11" s="53"/>
-      <c r="O11" s="53"/>
-      <c r="P11" s="53"/>
+        <v>4</v>
+      </c>
+      <c r="F11" s="66" t="s">
+        <v>308</v>
+      </c>
+      <c r="G11" s="76"/>
+      <c r="H11" s="76"/>
+      <c r="I11" s="76"/>
+      <c r="J11" s="77"/>
+      <c r="K11" s="77"/>
+      <c r="L11" s="77"/>
+      <c r="M11" s="77"/>
+      <c r="N11" s="76"/>
+      <c r="O11" s="76"/>
+      <c r="P11" s="76"/>
+      <c r="Q11" s="76"/>
+      <c r="R11" s="76"/>
     </row>
     <row r="12" spans="1:20" ht="24" customHeight="1">
       <c r="A12" s="49" t="s">
-        <v>328</v>
+        <v>316</v>
       </c>
       <c r="B12" s="49" t="s">
-        <v>329</v>
-      </c>
-      <c r="C12" s="50" t="s">
-        <v>330</v>
-      </c>
-      <c r="D12" s="50" t="s">
-        <v>331</v>
+        <v>317</v>
+      </c>
+      <c r="C12" s="81">
+        <v>46141</v>
+      </c>
+      <c r="D12" s="81">
+        <v>46169</v>
       </c>
       <c r="E12" s="50">
-        <v>3</v>
-      </c>
-      <c r="F12" s="51" t="s">
-        <v>310</v>
-      </c>
-      <c r="G12" s="53"/>
-      <c r="H12" s="53"/>
-      <c r="I12" s="53"/>
-      <c r="J12" s="52"/>
-      <c r="K12" s="53"/>
-      <c r="L12" s="53"/>
-      <c r="M12" s="53"/>
-      <c r="N12" s="53"/>
-      <c r="O12" s="53"/>
-      <c r="P12" s="53"/>
+        <v>4</v>
+      </c>
+      <c r="F12" s="66" t="s">
+        <v>308</v>
+      </c>
+      <c r="G12" s="76"/>
+      <c r="H12" s="76"/>
+      <c r="I12" s="76"/>
+      <c r="J12" s="77"/>
+      <c r="K12" s="77"/>
+      <c r="L12" s="77"/>
+      <c r="M12" s="77"/>
+      <c r="N12" s="76"/>
+      <c r="O12" s="76"/>
+      <c r="P12" s="76"/>
+      <c r="Q12" s="76"/>
+      <c r="R12" s="76"/>
     </row>
     <row r="13" spans="1:20" ht="24" customHeight="1">
       <c r="A13" s="49" t="s">
-        <v>328</v>
+        <v>316</v>
       </c>
       <c r="B13" s="49" t="s">
-        <v>332</v>
-      </c>
-      <c r="C13" s="50" t="s">
-        <v>333</v>
-      </c>
-      <c r="D13" s="50" t="s">
-        <v>334</v>
+        <v>318</v>
+      </c>
+      <c r="C13" s="81">
+        <v>46141</v>
+      </c>
+      <c r="D13" s="81">
+        <v>46169</v>
       </c>
       <c r="E13" s="50">
-        <v>2</v>
-      </c>
-      <c r="F13" s="51" t="s">
-        <v>310</v>
-      </c>
-      <c r="G13" s="53"/>
-      <c r="H13" s="53"/>
-      <c r="I13" s="53"/>
-      <c r="J13" s="52"/>
-      <c r="K13" s="53"/>
-      <c r="L13" s="53"/>
-      <c r="M13" s="53"/>
-      <c r="N13" s="53"/>
-      <c r="O13" s="53"/>
-      <c r="P13" s="53"/>
+        <v>4</v>
+      </c>
+      <c r="F13" s="66" t="s">
+        <v>308</v>
+      </c>
+      <c r="G13" s="76"/>
+      <c r="H13" s="76"/>
+      <c r="I13" s="76"/>
+      <c r="J13" s="77"/>
+      <c r="K13" s="77"/>
+      <c r="L13" s="77"/>
+      <c r="M13" s="77"/>
+      <c r="N13" s="76"/>
+      <c r="O13" s="76"/>
+      <c r="P13" s="76"/>
+      <c r="Q13" s="76"/>
+      <c r="R13" s="76"/>
     </row>
     <row r="14" spans="1:20" ht="24" customHeight="1">
       <c r="A14" s="49" t="s">
-        <v>335</v>
+        <v>319</v>
       </c>
       <c r="B14" s="49" t="s">
-        <v>336</v>
-      </c>
-      <c r="C14" s="50" t="s">
-        <v>337</v>
-      </c>
-      <c r="D14" s="50" t="s">
-        <v>338</v>
+        <v>320</v>
+      </c>
+      <c r="C14" s="81">
+        <v>46141</v>
+      </c>
+      <c r="D14" s="81">
+        <v>46169</v>
       </c>
       <c r="E14" s="50">
-        <v>1</v>
-      </c>
-      <c r="F14" s="51" t="s">
-        <v>310</v>
-      </c>
-      <c r="G14" s="53"/>
-      <c r="H14" s="53"/>
-      <c r="I14" s="53"/>
-      <c r="J14" s="52"/>
-      <c r="K14" s="53"/>
-      <c r="L14" s="53"/>
-      <c r="M14" s="53"/>
-      <c r="N14" s="53"/>
-      <c r="O14" s="53"/>
-      <c r="P14" s="53"/>
+        <v>4</v>
+      </c>
+      <c r="F14" s="66" t="s">
+        <v>308</v>
+      </c>
+      <c r="G14" s="76"/>
+      <c r="H14" s="76"/>
+      <c r="I14" s="76"/>
+      <c r="J14" s="77"/>
+      <c r="K14" s="77"/>
+      <c r="L14" s="77"/>
+      <c r="M14" s="77"/>
+      <c r="N14" s="76"/>
+      <c r="O14" s="76"/>
+      <c r="P14" s="76"/>
+      <c r="Q14" s="76"/>
+      <c r="R14" s="76"/>
     </row>
     <row r="15" spans="1:20" ht="24" customHeight="1">
       <c r="A15" s="49" t="s">
-        <v>335</v>
+        <v>319</v>
       </c>
       <c r="B15" s="49" t="s">
-        <v>339</v>
-      </c>
-      <c r="C15" s="50" t="s">
-        <v>340</v>
-      </c>
-      <c r="D15" s="50" t="s">
-        <v>341</v>
+        <v>321</v>
+      </c>
+      <c r="C15" s="81">
+        <v>46141</v>
+      </c>
+      <c r="D15" s="81">
+        <v>46169</v>
       </c>
       <c r="E15" s="50">
-        <v>1</v>
-      </c>
-      <c r="F15" s="51" t="s">
-        <v>310</v>
-      </c>
-      <c r="G15" s="53"/>
-      <c r="H15" s="53"/>
-      <c r="I15" s="53"/>
-      <c r="J15" s="52"/>
-      <c r="K15" s="53"/>
-      <c r="L15" s="53"/>
-      <c r="M15" s="53"/>
-      <c r="N15" s="53"/>
-      <c r="O15" s="53"/>
-      <c r="P15" s="53"/>
+        <v>4</v>
+      </c>
+      <c r="F15" s="66" t="s">
+        <v>308</v>
+      </c>
+      <c r="G15" s="76"/>
+      <c r="H15" s="76"/>
+      <c r="I15" s="76"/>
+      <c r="J15" s="77"/>
+      <c r="K15" s="77"/>
+      <c r="L15" s="77"/>
+      <c r="M15" s="77"/>
+      <c r="N15" s="76"/>
+      <c r="O15" s="76"/>
+      <c r="P15" s="76"/>
+      <c r="Q15" s="76"/>
+      <c r="R15" s="76"/>
     </row>
     <row r="16" spans="1:20" ht="24" customHeight="1">
       <c r="A16" s="49" t="s">
-        <v>335</v>
+        <v>319</v>
       </c>
       <c r="B16" s="49" t="s">
-        <v>342</v>
-      </c>
-      <c r="C16" s="50" t="s">
-        <v>343</v>
-      </c>
-      <c r="D16" s="50" t="s">
-        <v>344</v>
+        <v>322</v>
+      </c>
+      <c r="C16" s="81">
+        <v>46141</v>
+      </c>
+      <c r="D16" s="81">
+        <v>46169</v>
       </c>
       <c r="E16" s="50">
-        <v>1</v>
-      </c>
-      <c r="F16" s="51" t="s">
-        <v>310</v>
-      </c>
-      <c r="G16" s="53"/>
-      <c r="H16" s="53"/>
-      <c r="J16" s="52"/>
-      <c r="K16" s="53"/>
-      <c r="L16" s="53"/>
+        <v>4</v>
+      </c>
+      <c r="F16" s="66" t="s">
+        <v>308</v>
+      </c>
+      <c r="G16" s="76"/>
+      <c r="H16" s="76"/>
+      <c r="I16" s="76"/>
+      <c r="J16" s="77"/>
+      <c r="K16" s="77"/>
+      <c r="L16" s="77"/>
+      <c r="M16" s="77"/>
+      <c r="N16" s="76"/>
+      <c r="O16" s="76"/>
+      <c r="P16" s="76"/>
+      <c r="Q16" s="76"/>
+      <c r="R16" s="76"/>
     </row>
     <row r="17" spans="1:21" ht="24" customHeight="1">
       <c r="A17" s="49" t="s">
-        <v>335</v>
+        <v>319</v>
       </c>
       <c r="B17" s="49" t="s">
-        <v>345</v>
-      </c>
-      <c r="C17" s="50" t="s">
-        <v>341</v>
-      </c>
-      <c r="D17" s="50" t="s">
-        <v>346</v>
-      </c>
+        <v>323</v>
+      </c>
+      <c r="C17" s="81">
+        <v>46153</v>
+      </c>
+      <c r="D17" s="81"/>
       <c r="E17" s="50">
-        <v>2</v>
-      </c>
-      <c r="F17" s="54" t="s">
-        <v>347</v>
-      </c>
-      <c r="G17" s="53"/>
-      <c r="H17" s="53"/>
-      <c r="I17" s="53"/>
-      <c r="J17" s="55"/>
-      <c r="K17" s="55"/>
-      <c r="L17" s="53"/>
+        <v>4</v>
+      </c>
+      <c r="F17" s="67" t="s">
+        <v>324</v>
+      </c>
+      <c r="G17" s="76"/>
+      <c r="H17" s="76"/>
+      <c r="I17" s="76"/>
+      <c r="J17" s="76"/>
+      <c r="K17" s="78"/>
+      <c r="L17" s="78"/>
+      <c r="M17" s="78"/>
+      <c r="N17" s="78"/>
+      <c r="O17" s="76"/>
+      <c r="P17" s="76"/>
+      <c r="Q17" s="76"/>
+      <c r="R17" s="76"/>
     </row>
     <row r="18" spans="1:21" ht="24" customHeight="1">
       <c r="A18" s="49" t="s">
-        <v>335</v>
+        <v>319</v>
       </c>
       <c r="B18" s="49" t="s">
-        <v>348</v>
-      </c>
-      <c r="C18" s="50" t="s">
-        <v>344</v>
-      </c>
-      <c r="D18" s="50" t="s">
-        <v>349</v>
-      </c>
+        <v>325</v>
+      </c>
+      <c r="C18" s="81">
+        <v>46153</v>
+      </c>
+      <c r="D18" s="81"/>
       <c r="E18" s="50">
-        <v>1</v>
-      </c>
-      <c r="F18" s="54" t="s">
-        <v>347</v>
-      </c>
-      <c r="G18" s="53"/>
-      <c r="H18" s="53"/>
-      <c r="I18" s="53"/>
-      <c r="J18" s="55"/>
-      <c r="K18" s="55"/>
-      <c r="L18" s="53"/>
-      <c r="U18" s="80"/>
+        <v>4</v>
+      </c>
+      <c r="F18" s="67" t="s">
+        <v>324</v>
+      </c>
+      <c r="G18" s="76"/>
+      <c r="H18" s="76"/>
+      <c r="I18" s="76"/>
+      <c r="J18" s="76"/>
+      <c r="K18" s="78"/>
+      <c r="L18" s="78"/>
+      <c r="M18" s="78"/>
+      <c r="N18" s="78"/>
+      <c r="O18" s="76"/>
+      <c r="P18" s="76"/>
+      <c r="Q18" s="76"/>
+      <c r="R18" s="76"/>
+      <c r="U18" s="65"/>
     </row>
     <row r="19" spans="1:21" ht="24" customHeight="1">
       <c r="A19" s="49" t="s">
-        <v>335</v>
+        <v>319</v>
       </c>
       <c r="B19" s="49" t="s">
-        <v>350</v>
-      </c>
-      <c r="C19" s="50" t="s">
-        <v>351</v>
-      </c>
-      <c r="D19" s="50" t="s">
-        <v>352</v>
-      </c>
+        <v>326</v>
+      </c>
+      <c r="C19" s="81"/>
+      <c r="D19" s="81"/>
       <c r="E19" s="50">
         <v>1</v>
       </c>
-      <c r="F19" s="56" t="s">
-        <v>353</v>
-      </c>
-      <c r="G19" s="53"/>
-      <c r="H19" s="53"/>
-      <c r="I19" s="53"/>
-      <c r="J19" s="57"/>
-      <c r="K19" s="57"/>
-      <c r="L19" s="53"/>
+      <c r="F19" s="68" t="s">
+        <v>327</v>
+      </c>
+      <c r="G19" s="76"/>
+      <c r="H19" s="76"/>
+      <c r="I19" s="76"/>
+      <c r="J19" s="76"/>
+      <c r="K19" s="76"/>
+      <c r="L19" s="76"/>
+      <c r="M19" s="79"/>
+      <c r="N19" s="78"/>
+      <c r="O19" s="76"/>
+      <c r="P19" s="76"/>
+      <c r="Q19" s="76"/>
+      <c r="R19" s="76"/>
     </row>
     <row r="20" spans="1:21" ht="24" customHeight="1">
       <c r="A20" s="49" t="s">
-        <v>335</v>
+        <v>319</v>
       </c>
       <c r="B20" s="49" t="s">
-        <v>354</v>
-      </c>
-      <c r="C20" s="50" t="s">
-        <v>355</v>
-      </c>
-      <c r="D20" s="50" t="s">
-        <v>356</v>
-      </c>
+        <v>328</v>
+      </c>
+      <c r="C20" s="81"/>
+      <c r="D20" s="81"/>
       <c r="E20" s="50">
         <v>2</v>
       </c>
-      <c r="F20" s="56" t="s">
-        <v>353</v>
-      </c>
-      <c r="G20" s="53"/>
-      <c r="H20" s="53"/>
-      <c r="I20" s="53"/>
-      <c r="J20" s="57"/>
-      <c r="K20" s="57"/>
-      <c r="L20" s="53"/>
+      <c r="F20" s="68" t="s">
+        <v>327</v>
+      </c>
+      <c r="G20" s="76"/>
+      <c r="H20" s="76"/>
+      <c r="I20" s="76"/>
+      <c r="J20" s="76"/>
+      <c r="K20" s="76"/>
+      <c r="L20" s="76"/>
+      <c r="M20" s="79"/>
+      <c r="N20" s="79"/>
+      <c r="O20" s="76"/>
+      <c r="P20" s="76"/>
+      <c r="Q20" s="76"/>
+      <c r="R20" s="76"/>
     </row>
     <row r="21" spans="1:21" ht="24" customHeight="1">
       <c r="A21" s="49" t="s">
-        <v>357</v>
+        <v>329</v>
       </c>
       <c r="B21" s="49" t="s">
-        <v>358</v>
-      </c>
-      <c r="C21" s="50" t="s">
-        <v>352</v>
-      </c>
-      <c r="D21" s="50" t="s">
-        <v>359</v>
-      </c>
+        <v>330</v>
+      </c>
+      <c r="C21" s="81"/>
+      <c r="D21" s="81"/>
       <c r="E21" s="50">
         <v>1</v>
       </c>
-      <c r="F21" s="56" t="s">
-        <v>353</v>
-      </c>
-      <c r="G21" s="53"/>
-      <c r="H21" s="53"/>
-      <c r="I21" s="53"/>
-      <c r="J21" s="53"/>
-      <c r="K21" s="57"/>
-      <c r="L21" s="57"/>
+      <c r="F21" s="68" t="s">
+        <v>327</v>
+      </c>
+      <c r="G21" s="76"/>
+      <c r="H21" s="76"/>
+      <c r="I21" s="76"/>
+      <c r="J21" s="76"/>
+      <c r="K21" s="76"/>
+      <c r="L21" s="76"/>
+      <c r="M21" s="76"/>
+      <c r="N21" s="79"/>
+      <c r="O21" s="79"/>
+      <c r="P21" s="76"/>
+      <c r="Q21" s="76"/>
+      <c r="R21" s="76"/>
     </row>
     <row r="22" spans="1:21" ht="24" customHeight="1">
       <c r="A22" s="49" t="s">
-        <v>357</v>
+        <v>329</v>
       </c>
       <c r="B22" s="49" t="s">
-        <v>360</v>
-      </c>
-      <c r="C22" s="50" t="s">
-        <v>361</v>
-      </c>
-      <c r="D22" s="50" t="s">
-        <v>362</v>
-      </c>
+        <v>331</v>
+      </c>
+      <c r="C22" s="81"/>
+      <c r="D22" s="81"/>
       <c r="E22" s="50">
         <v>1</v>
       </c>
-      <c r="F22" s="56" t="s">
-        <v>353</v>
-      </c>
-      <c r="G22" s="53"/>
-      <c r="H22" s="53"/>
-      <c r="I22" s="53"/>
-      <c r="J22" s="53"/>
-      <c r="K22" s="57"/>
-      <c r="L22" s="57"/>
+      <c r="F22" s="68" t="s">
+        <v>327</v>
+      </c>
+      <c r="G22" s="76"/>
+      <c r="H22" s="76"/>
+      <c r="I22" s="76"/>
+      <c r="J22" s="76"/>
+      <c r="K22" s="76"/>
+      <c r="L22" s="76"/>
+      <c r="M22" s="76"/>
+      <c r="N22" s="79"/>
+      <c r="O22" s="79"/>
+      <c r="P22" s="76"/>
+      <c r="Q22" s="76"/>
+      <c r="R22" s="76"/>
     </row>
     <row r="23" spans="1:21" ht="24" customHeight="1">
       <c r="A23" s="49" t="s">
-        <v>357</v>
+        <v>329</v>
       </c>
       <c r="B23" s="49" t="s">
-        <v>363</v>
-      </c>
-      <c r="C23" s="50" t="s">
-        <v>359</v>
-      </c>
-      <c r="D23" s="50" t="s">
-        <v>364</v>
-      </c>
+        <v>332</v>
+      </c>
+      <c r="C23" s="81"/>
+      <c r="D23" s="81"/>
       <c r="E23" s="50">
         <v>1</v>
       </c>
-      <c r="F23" s="56" t="s">
-        <v>353</v>
-      </c>
-      <c r="G23" s="53"/>
-      <c r="H23" s="53"/>
-      <c r="I23" s="53"/>
-      <c r="J23" s="53"/>
-      <c r="K23" s="53"/>
-      <c r="L23" s="57"/>
+      <c r="F23" s="68" t="s">
+        <v>327</v>
+      </c>
+      <c r="G23" s="76"/>
+      <c r="H23" s="76"/>
+      <c r="I23" s="76"/>
+      <c r="J23" s="76"/>
+      <c r="K23" s="76"/>
+      <c r="L23" s="76"/>
+      <c r="M23" s="76"/>
+      <c r="N23" s="76"/>
+      <c r="O23" s="79"/>
+      <c r="P23" s="76"/>
+      <c r="Q23" s="76"/>
+      <c r="R23" s="76"/>
     </row>
     <row r="24" spans="1:21" ht="24" customHeight="1">
       <c r="A24" s="49" t="s">
-        <v>357</v>
+        <v>329</v>
       </c>
       <c r="B24" s="49" t="s">
-        <v>365</v>
-      </c>
-      <c r="C24" s="50" t="s">
-        <v>362</v>
-      </c>
-      <c r="D24" s="50" t="s">
-        <v>366</v>
-      </c>
+        <v>333</v>
+      </c>
+      <c r="C24" s="81"/>
+      <c r="D24" s="81"/>
       <c r="E24" s="50">
         <v>1</v>
       </c>
-      <c r="F24" s="56" t="s">
-        <v>353</v>
-      </c>
-      <c r="G24" s="53"/>
-      <c r="H24" s="53"/>
-      <c r="I24" s="53"/>
-      <c r="J24" s="53"/>
-      <c r="K24" s="53"/>
-      <c r="L24" s="57"/>
+      <c r="F24" s="68" t="s">
+        <v>327</v>
+      </c>
+      <c r="G24" s="70"/>
+      <c r="H24" s="70"/>
+      <c r="I24" s="70"/>
+      <c r="J24" s="70"/>
+      <c r="K24" s="70"/>
+      <c r="L24" s="70"/>
+      <c r="M24" s="70"/>
+      <c r="N24" s="70"/>
+      <c r="O24" s="80"/>
+      <c r="P24" s="70"/>
+      <c r="Q24" s="70"/>
+      <c r="R24" s="70"/>
     </row>
     <row r="27" spans="1:21">
       <c r="A27" s="48" t="s">
-        <v>367</v>
-      </c>
-      <c r="B27" s="52"/>
+        <v>334</v>
+      </c>
+      <c r="B27" s="51"/>
       <c r="C27" s="48" t="s">
-        <v>310</v>
-      </c>
-      <c r="D27" s="55"/>
+        <v>308</v>
+      </c>
+      <c r="D27" s="52"/>
       <c r="E27" s="48" t="s">
-        <v>347</v>
-      </c>
-      <c r="F27" s="57"/>
+        <v>324</v>
+      </c>
+      <c r="F27" s="53"/>
       <c r="G27" s="48" t="s">
-        <v>353</v>
+        <v>327</v>
       </c>
     </row>
   </sheetData>
@@ -13558,6 +13633,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <TaxCatchAll xmlns="68f69d94-ca7b-455f-a2e9-4b6b05bed5cf" xsi:nil="true"/>
@@ -13566,15 +13650,6 @@
     </lcf76f155ced4ddcb4097134ff3c332f>
   </documentManagement>
 </p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -13813,11 +13888,11 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{46626F29-F59B-4A91-8F55-0DF315CA6A8D}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D02AA35A-4357-4E53-B26D-4F99101B638F}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D02AA35A-4357-4E53-B26D-4F99101B638F}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{46626F29-F59B-4A91-8F55-0DF315CA6A8D}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>